<commit_message>
feat: update logistics optimizer with VRP backhauling details, presentation assets, and scratch scripts
</commit_message>
<xml_diff>
--- a/FINAL_SUBMISSION_TFM/results_analysis/resumen_comparativo_modalidades.xlsx
+++ b/FINAL_SUBMISSION_TFM/results_analysis/resumen_comparativo_modalidades.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Modalidad</t>
   </si>
@@ -25,10 +25,16 @@
     <t>Nº EV</t>
   </si>
   <si>
+    <t>TCO Activos (VAN) (€)</t>
+  </si>
+  <si>
+    <t>TCO Personal (VAN) (€)</t>
+  </si>
+  <si>
+    <t>TCO TOTAL OPERACIÓN (€)</t>
+  </si>
+  <si>
     <t>Valor Residual Total (€)</t>
-  </si>
-  <si>
-    <t>TCO Total (VAN) (€)</t>
   </si>
   <si>
     <t>Coste Medio (€/km)</t>
@@ -398,10 +404,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -420,10 +426,16 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>33</v>
@@ -432,18 +444,24 @@
         <v>18</v>
       </c>
       <c r="D2">
+        <v>16817858.69845043</v>
+      </c>
+      <c r="E2">
+        <v>7046848.23672479</v>
+      </c>
+      <c r="F2">
+        <v>23864706.93517522</v>
+      </c>
+      <c r="G2">
         <v>3186000</v>
       </c>
-      <c r="E2">
-        <v>16817858.69845043</v>
-      </c>
-      <c r="F2">
-        <v>0.5073260542518984</v>
+      <c r="H2">
+        <v>0.7199006616945768</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>33</v>
@@ -452,18 +470,24 @@
         <v>18</v>
       </c>
       <c r="D3">
+        <v>16058316.53976777</v>
+      </c>
+      <c r="E3">
+        <v>7046848.23672479</v>
+      </c>
+      <c r="F3">
+        <v>23105164.77649257</v>
+      </c>
+      <c r="G3">
         <v>3186000</v>
       </c>
-      <c r="E3">
-        <v>16058316.53976777</v>
-      </c>
-      <c r="F3">
-        <v>0.4844137719386961</v>
+      <c r="H3">
+        <v>0.6969883793813746</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>33</v>
@@ -472,13 +496,19 @@
         <v>18</v>
       </c>
       <c r="D4">
+        <v>15670498.12156428</v>
+      </c>
+      <c r="E4">
+        <v>7046848.23672479</v>
+      </c>
+      <c r="F4">
+        <v>22717346.35828907</v>
+      </c>
+      <c r="G4">
         <v>0</v>
       </c>
-      <c r="E4">
-        <v>15670498.12156428</v>
-      </c>
-      <c r="F4">
-        <v>0.4727148754619692</v>
+      <c r="H4">
+        <v>0.6852894829046476</v>
       </c>
     </row>
   </sheetData>

</xml_diff>